<commit_message>
changed repetitive search for posting_ids when looking for corrected additional tests for margin & novelty
</commit_message>
<xml_diff>
--- a/test_results.xlsx
+++ b/test_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="51.21875" customWidth="1" min="1" max="1"/>
@@ -579,6 +579,76 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>training_strat= retrain, l=3, corrected_weights = 100, corrected_saved = True, strategy = entropy</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2059, Recall: 0.9392, TP: 535, FP: 2044, TN: 48505, FN: 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2077, Recall: 0.9497, TP: 535, FP: 1971, TN: 48578, FN: 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Iteration: 3, Precision: 0.2082, Recall: 0.9566, TP: 550, FP: 1911, TN: 48638, FN: 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>training_strat= retrain, l=3, corrected_weights = 100, corrected_saved = True, strategy = entropy</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2059, Recall: 0.9392, TP: 535, FP: 2044, TN: 48505, FN: 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2077, Recall: 0.9497, TP: 535, FP: 1971, TN: 48578, FN: 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Iteration: 3, Precision: 0.2082, Recall: 0.9566, TP: 550, FP: 1911, TN: 48638, FN: 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor greedy algorithm and enhance retraining process with new state management and uncertainty scoring
</commit_message>
<xml_diff>
--- a/test_results.xlsx
+++ b/test_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Balda\PycharmProjects\AD2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E79D4C5-656C-441A-A89D-6A5083B7B2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16492D2-C03F-4A63-9601-9F8064F83FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,11 @@
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
   <si>
     <t>retrain, l=10, corrected_weights = 10, corrected_safed = False, strategy = entropy</t>
   </si>
@@ -35,6 +34,9 @@
     <t>Iteration: 10, Precision: 0.2070, Recall: 0.9688, TP: 556, FP: 2052, TN: 48497, FN: 20</t>
   </si>
   <si>
+    <t>================================================================================</t>
+  </si>
+  <si>
     <t>retrain, l=10, corrected_weights = 10, corrected_saved = True, strategy = entropy</t>
   </si>
   <si>
@@ -59,9 +61,6 @@
     <t>Iteration: 100, Precision: 0.2334, Recall: 1.0000, TP: 574, FP: 1699, TN: 48850, FN: 2</t>
   </si>
   <si>
-    <t>================================================================================</t>
-  </si>
-  <si>
     <t>retrain, l=100, corrected_weights = 100, corrected_saved = False, strategy = entropy</t>
   </si>
   <si>
@@ -84,6 +83,60 @@
   </si>
   <si>
     <t>'================================================================================</t>
+  </si>
+  <si>
+    <t>[2026-08-07 10:40:23] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = entropy, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = True</t>
+  </si>
+  <si>
+    <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000</t>
+  </si>
+  <si>
+    <t>Iteration: 2, Precision: 0.2069, Recall: 0.9601, TP: 539, FP: 2043, TN: 48506, FN: 37, type=new_center, centers=2, covered=2, cum_direct=2, flipped=1, prop_acc=1.0000, T=0.5000</t>
+  </si>
+  <si>
+    <t>[2026-08-07 10:41:36] | training_strat= retrain, l=1, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = False, greedy_T = None, compute_shap = False, skip_retrain_on_skip = False</t>
+  </si>
+  <si>
+    <t>Iteration: 1, Precision: 0.2059, Recall: 0.9392, TP: 535, FP: 2044, TN: 48505, FN: 41, Misspredicted: 4</t>
+  </si>
+  <si>
+    <t>[2026-08-05 05:16:34] | training_strat= retrain, l=50, corrected_weights = 100, corrected_saved = True, strategy = entropy, greedy_batching = True</t>
+  </si>
+  <si>
+    <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.1980</t>
+  </si>
+  <si>
+    <t>Iteration: 26, Precision: 0.2081, Recall: 0.9757, TP: 562, FP: 2063, TN: 48486, FN: 14, type=new_center, centers=26, covered=62, cum_direct=26, flipped=0, prop_acc=1.0000, T=0.1980</t>
+  </si>
+  <si>
+    <t>Iteration: 50, Precision: 0.2087, Recall: 0.9757, TP: 562, FP: 2056, TN: 48493, FN: 14, type=new_center, centers=50, covered=113, cum_direct=50, flipped=0, prop_acc=1.0000, T=0.1980</t>
+  </si>
+  <si>
+    <t>[2026-08-05 05:44:12] | training_strat= retrain, l=50, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True</t>
+  </si>
+  <si>
+    <t>[2026-08-05 06:16:25] | training_strat= retrain, l=50, corrected_weights = 100, corrected_saved = True, strategy = entropy, greedy_batching = True</t>
+  </si>
+  <si>
+    <t>Iteration: 26, Precision: 0.2124, Recall: 0.9722, TP: 559, FP: 1974, TN: 48575, FN: 17, type=new_center, centers=26, covered=220, cum_direct=26, flipped=0, prop_acc=1.0000, T=0.5000</t>
+  </si>
+  <si>
+    <t>Iteration: 50, Precision: 0.2140, Recall: 0.9774, TP: 563, FP: 1939, TN: 48610, FN: 13, type=new_center, centers=50, covered=298, cum_direct=50, flipped=2, prop_acc=1.0000, T=0.5000</t>
+  </si>
+  <si>
+    <t>[2026-08-05 06:44:01] | training_strat= retrain, l=50, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True</t>
+  </si>
+  <si>
+    <t>[2026-08-05 11:43:48] | training_strat= retrain, l=500, corrected_weights = 100, corrected_saved = True, strategy = entropy, greedy_batching = True</t>
+  </si>
+  <si>
+    <t>Iteration: 251, Precision: 0.2640, Recall: 1.0000, TP: 576, FP: 1602, TN: 48947, FN: 0, type=new_center, centers=251, covered=883, cum_direct=251, flipped=1, prop_acc=1.0000, T=0.5000</t>
+  </si>
+  <si>
+    <t>Iteration: 500, Precision: 0.3408, Recall: 1.0000, TP: 576, FP: 1102, TN: 49447, FN: 0, type=new_center, centers=486, covered=1460, cum_direct=500, flipped=8, prop_acc=1.0000, T=0.5000</t>
+  </si>
+  <si>
+    <t>[2026-08-05 16:44:15] | training_strat= retrain, l=500, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True</t>
   </si>
 </sst>
 </file>
@@ -119,9 +172,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -424,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.28515625" customWidth="1"/>
@@ -452,57 +506,57 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -527,7 +581,7 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
@@ -537,22 +591,22 @@
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
@@ -562,7 +616,7 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
@@ -587,7 +641,7 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
@@ -602,6 +656,191 @@
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add distance-weighted labels and density-targeted selection
- greedy.py: add neighbor_density computation (radius=T), selection_mode
  parameter for uncertainty_density selection, cache nearest_dist in state
- main.py: add prop_weight_mode (uniform/linear_decay/gaussian_decay) for
  distance-decayed propagation weights, selection_mode forwarding
- kittyboost.py: add sample_weights parameter for per-case weight arrays
- Add AGENTS.md and PROJECT_CONTEXT.md for session continuity
</commit_message>
<xml_diff>
--- a/test_results.xlsx
+++ b/test_results.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
@@ -45,9 +45,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -414,10 +416,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A94"/>
+  <dimension ref="A1:A139"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col width="51.28515625" customWidth="1" style="2" min="1" max="1"/>
+    <col width="51.28515625" customWidth="1" style="4" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -997,82 +999,397 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>[2026-08-17 13:44:42] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['features_all']</t>
+          <t>[2026-08-09 09:30:06] | training_strat= retrain, l=50, corrected_weights = 100, corrected_saved = True, strategy = entropy, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = True</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+          <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Iteration: 2, Precision: 0.2069, Recall: 0.9601, TP: 539, FP: 2043, TN: 48506, FN: 37, type=new_center, centers=2, covered=2, cum_direct=2, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+          <t>Iteration: 26, Precision: 0.2124, Recall: 0.9722, TP: 559, FP: 1974, TN: 48575, FN: 17, type=new_center, centers=26, covered=220, cum_direct=26, flipped=0, prop_acc=1.0000, T=0.5000</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>'================================================================================</t>
+          <t>Iteration: 50, Precision: 0.2140, Recall: 0.9774, TP: 563, FP: 1939, TN: 48610, FN: 13, type=new_center, centers=50, covered=298, cum_direct=50, flipped=2, prop_acc=1.0000, T=0.5000</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>[2026-08-17 13:47:00] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_all']</t>
+          <t>'================================================================================</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Iteration: 1, Precision: 0.2055, Recall: 0.9444, TP: 549, FP: 2116, TN: 48433, FN: 27, type=new_center, centers=1, covered=4, cum_direct=1, flipped=4, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+          <t>[2026-08-09 11:17:03] | training_strat= retrain, l=500, corrected_weights = 100, corrected_saved = True, strategy = novelty, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = True</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Iteration: 2, Precision: 0.2066, Recall: 0.9549, TP: 555, FP: 2127, TN: 48422, FN: 21, type=new_center, centers=2, covered=6, cum_direct=2, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+          <t>Iteration: 1, Precision: 0.2054, Recall: 0.9462, TP: 547, FP: 2111, TN: 48438, FN: 29, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>'================================================================================</t>
+          <t>Iteration: 251, Precision: 0.1694, Recall: 0.9896, TP: 565, FP: 2442, TN: 48107, FN: 11, type=skip (retrain skipped)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>[2026-08-17 13:49:28] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['features_raw', 'shap_all']</t>
+          <t>Iteration: 500, Precision: 0.1515, Recall: 1.0000, TP: 558, FP: 2545, TN: 48004, FN: 18, type=new_center, centers=443, covered=515, cum_direct=500, flipped=1, prop_acc=1.0000, T=0.5000</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=131</t>
+          <t>'================================================================================</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Iteration: 2, Precision: 0.2069, Recall: 0.9601, TP: 539, FP: 2043, TN: 48506, FN: 37, type=new_center, centers=2, covered=2, cum_direct=2, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=131</t>
+          <t>[2026-08-17 13:44:42] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['features_all']</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2069, Recall: 0.9601, TP: 539, FP: 2043, TN: 48506, FN: 37, type=new_center, centers=2, covered=2, cum_direct=2, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>[2026-08-17 13:47:00] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_all']</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2055, Recall: 0.9444, TP: 549, FP: 2116, TN: 48433, FN: 27, type=new_center, centers=1, covered=4, cum_direct=1, flipped=4, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2066, Recall: 0.9549, TP: 555, FP: 2127, TN: 48422, FN: 21, type=new_center, centers=2, covered=6, cum_direct=2, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>[2026-08-17 13:49:28] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['features_raw', 'shap_all']</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=131</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2069, Recall: 0.9601, TP: 539, FP: 2043, TN: 48506, FN: 37, type=new_center, centers=2, covered=2, cum_direct=2, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=131</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>[2026-08-17 20:45:08] | training_strat= retrain, l=500, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['features_all', 'shap_all']</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2056, Recall: 0.9479, TP: 525, FP: 1997, TN: 48552, FN: 51, type=new_center, centers=1, covered=1, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=158</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Iteration: 251, Precision: 0.2316, Recall: 1.0000, TP: 576, FP: 1877, TN: 48672, FN: 0, type=new_center, centers=251, covered=403, cum_direct=251, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=158</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Iteration: 500, Precision: 0.2753, Recall: 1.0000, TP: 576, FP: 1502, TN: 49047, FN: 0, type=new_center, centers=500, covered=925, cum_direct=500, flipped=2, prop_acc=1.0000, T=0.5000, prop_dims=158</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>[2026-08-21 12:08:24] | training_strat= retrain, l=500, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['features_raw']</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2057, Recall: 0.9479, TP: 550, FP: 2116, TN: 48433, FN: 26, type=new_center, centers=1, covered=9, cum_direct=1, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=52</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Iteration: 251, Precision: 0.3049, Recall: 1.0000, TP: 571, FP: 1163, TN: 49386, FN: 5, type=new_center, centers=248, covered=18882, cum_direct=251, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=52</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Iteration: 500, Precision: 0.4630, Recall: 1.0000, TP: 572, FP: 641, TN: 49908, FN: 4, type=new_center, centers=487, covered=22269, cum_direct=500, flipped=0, prop_acc=0.9996, T=0.5000, prop_dims=52</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>[2026-08-21 16:18:21] | training_strat= retrain, l=500, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_all']</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2055, Recall: 0.9444, TP: 549, FP: 2116, TN: 48433, FN: 27, type=new_center, centers=1, covered=4, cum_direct=1, flipped=4, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Iteration: 251, Precision: 0.2389, Recall: 1.0000, TP: 576, FP: 1828, TN: 48721, FN: 0, type=new_center, centers=251, covered=562, cum_direct=251, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Iteration: 500, Precision: 0.3119, Recall: 1.0000, TP: 576, FP: 1256, TN: 49293, FN: 0, type=new_center, centers=497, covered=1552, cum_direct=500, flipped=1, prop_acc=0.9987, T=0.5000, prop_dims=79</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>[2026-08-24 22:24:34] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_raw'], prop_weight_mode = uniform, selection_mode = uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2055, Recall: 0.9444, TP: 549, FP: 2116, TN: 48433, FN: 27, type=new_center, centers=1, covered=4, cum_direct=1, flipped=4, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=uniform, sel_mode=uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2066, Recall: 0.9549, TP: 555, FP: 2127, TN: 48422, FN: 21, type=new_center, centers=2, covered=6, cum_direct=2, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=uniform, sel_mode=uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>[2026-08-24 22:28:34] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_raw'], prop_weight_mode = uniform, selection_mode = uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2055, Recall: 0.9444, TP: 549, FP: 2116, TN: 48433, FN: 27, type=new_center, centers=1, covered=4, cum_direct=1, flipped=4, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=uniform, sel_mode=uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2066, Recall: 0.9549, TP: 555, FP: 2127, TN: 48422, FN: 21, type=new_center, centers=2, covered=6, cum_direct=2, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=uniform, sel_mode=uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>[2026-08-24 22:31:06] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_raw'], prop_weight_mode = linear_decay, selection_mode = uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2055, Recall: 0.9444, TP: 531, FP: 2028, TN: 48521, FN: 45, type=new_center, centers=1, covered=4, cum_direct=1, flipped=4, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=linear_decay, sel_mode=uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2068, Recall: 0.9566, TP: 542, FP: 2061, TN: 48488, FN: 34, type=new_center, centers=2, covered=19, cum_direct=2, flipped=1, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=linear_decay, sel_mode=uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>[2026-08-24 22:33:21] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_raw'], prop_weight_mode = uniform, selection_mode = uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2055, Recall: 0.9462, TP: 551, FP: 2127, TN: 48422, FN: 25, type=new_center, centers=1, covered=17, cum_direct=1, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=uniform, sel_mode=uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2067, Recall: 0.9601, TP: 543, FP: 2062, TN: 48487, FN: 33, type=new_center, centers=2, covered=25, cum_direct=2, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=uniform, sel_mode=uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>[2026-08-24 22:35:42] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_raw'], prop_weight_mode = linear_decay, selection_mode = uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2063, Recall: 0.9497, TP: 547, FP: 2101, TN: 48448, FN: 29, type=new_center, centers=1, covered=17, cum_direct=1, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=linear_decay, sel_mode=uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2070, Recall: 0.9601, TP: 546, FP: 2072, TN: 48477, FN: 30, type=new_center, centers=2, covered=184, cum_direct=2, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=linear_decay, sel_mode=uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
         <is>
           <t>'================================================================================</t>
         </is>

</xml_diff>

<commit_message>
1. SHAP bedingt (kittyboost.py:78, main.py:182): shap_vals=None wenn kein shap_* im propagation_space. main.py:131 und greedy.py prüfen bereits auf None. 2. Matrix-Cache (greedy.py:101): Cache-Key = id(state["shap_vals"]). Da shap_vals nach jedem Retrain neu zugewiesen wird (main.py:100/67), wird der Cache automatisch bei SHAP-Update invalidiert. Sonst bleibt er stabil. 3. Density nur bei uncertainty_density (greedy.py:226): radius_neighbors_graph läuft nur noch bedarfsgerecht. M_density (Zeile 286) handhabt None bereits → loggt 0.0 bei uncertainty. 4. _prop_dims vektorisiert (greedy.py:133): ohne Matrix-Allokation, identische Dim-Berechnung. 5. .assign() in isolation_forest.py:54: funktionsäquivalent zu .copy() + Zuweisung.
</commit_message>
<xml_diff>
--- a/test_results.xlsx
+++ b/test_results.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A139"/>
+  <dimension ref="A1:A143"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="51.28515625" customWidth="1" style="4" min="1" max="1"/>
@@ -1395,6 +1395,34 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>[2026-09-05 17:11:50] | training_strat= retrain, l=2, corrected_weights = 100, corrected_saved = True, strategy = margin, greedy_batching = True, greedy_T = 0.5, compute_shap = False, skip_retrain_on_skip = False, propagation_space = ['shap_raw'], prop_weight_mode = linear_decay, selection_mode = uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Iteration: 1, Precision: 0.2063, Recall: 0.9497, TP: 547, FP: 2101, TN: 48448, FN: 29, type=new_center, centers=1, covered=17, cum_direct=1, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=linear_decay, sel_mode=uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Iteration: 2, Precision: 0.2070, Recall: 0.9601, TP: 546, FP: 2072, TN: 48477, FN: 30, type=new_center, centers=2, covered=184, cum_direct=2, flipped=0, prop_acc=1.0000, T=0.5000, prop_dims=52, weight_mode=linear_decay, sel_mode=uncertainty_density</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>'================================================================================</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>